<commit_message>
Revisión integral: reportes de rotación, cobros y descripciones de productos
- Reporte de ventas con los cinco más vendidos; inventario con baja rotación (pantalla, PDF y hoja de Excel)
- Registrar pago: el monto se llena con el total en la moneda del método
- El cliente ve «Estamos verificando tu pago» mientras se revisa
- Descripción breve de para qué sirve cada producto (tarjeta y ficha)
- Datos de prueba con los cuatro reportes del mes; 128 pruebas aprobadas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/seeders/catalogo/productos.xlsx
+++ b/database/seeders/catalogo/productos.xlsx
@@ -60,7 +60,7 @@
     <t>Marchesan Tatu</t>
   </si>
   <si>
-    <t>Rotativa Tatu modelo 3400, color azul.</t>
+    <t>Implemento que se acopla al tractor para cortar pasto, maleza y rastrojo en potreros y cultivos. Modelo 3400, color azul, original Tatu.</t>
   </si>
   <si>
     <t>0104090017C.jpeg</t>
@@ -78,7 +78,7 @@
     <t>Rotativas Tatu</t>
   </si>
   <si>
-    <t>Par de cuchillas originales Tatu.</t>
+    <t>Cuchillas que hacen el corte en la rotativa. Se cambian en par para mantener el rotor equilibrado y un corte parejo. Originales Tatu.</t>
   </si>
   <si>
     <t>0501052742R.jpeg</t>
@@ -93,7 +93,7 @@
     <t>Transmisión y cardanes</t>
   </si>
   <si>
-    <t>Conjunto de piñón y corona original Tatu.</t>
+    <t>Engranajes de la caja de transmisión que llevan la fuerza del cardán al eje de corte. Se reemplazan juntos para que engranen bien. Original Tatu.</t>
   </si>
   <si>
     <t>0503060210R.jpeg</t>
@@ -108,7 +108,7 @@
     <t>Rastras Tatu</t>
   </si>
   <si>
-    <t>Disco dentado para rastra, 24 x 6 5/16, original Tatu.</t>
+    <t>Disco dentado que corta y voltea la tierra y los rastrojos al preparar el suelo para la siembra. Medida 24" x 6 5/16", original Tatu.</t>
   </si>
   <si>
     <t>0602030250R.jpeg</t>
@@ -120,7 +120,7 @@
     <t>Tornillo para cuchilla</t>
   </si>
   <si>
-    <t>Tornillo de fijación para cuchilla de rotativa, original Tatu.</t>
+    <t>Fija la cuchilla al plato de la rotativa. Conviene cambiarlo junto con las cuchillas. Original Tatu.</t>
   </si>
   <si>
     <t>0501047573R.jpeg</t>
@@ -135,7 +135,7 @@
     <t>Colombo Aemco</t>
   </si>
   <si>
-    <t>Cardán completo Aemco, serie 330.</t>
+    <t>Eje que transmite la potencia de la toma de fuerza del tractor al implemento (rotativa, rastra, bomba). Serie 330, original Aemco.</t>
   </si>
   <si>
     <t>CC5002-3.jpeg</t>
@@ -147,7 +147,7 @@
     <t>Cardán completo cruceta 27 x 80</t>
   </si>
   <si>
-    <t>Cardán completo Aemco con cruceta 27 x 80.</t>
+    <t>Eje de transmisión completo que lleva la potencia de la toma de fuerza del tractor al implemento. Con cruceta 27 x 80, original Aemco.</t>
   </si>
   <si>
     <t>CC2051-11.jpeg</t>
@@ -159,7 +159,7 @@
     <t>Junta completa e/e 330</t>
   </si>
   <si>
-    <t>Junta completa estriado/estriado, serie 330.</t>
+    <t>Junta de cardán con los dos extremos estriados: une el cardán con la toma de fuerza y con el eje del implemento. Serie 330.</t>
   </si>
   <si>
     <t>CC565556.jpeg</t>
@@ -171,7 +171,7 @@
     <t>Yugo estriado 330</t>
   </si>
   <si>
-    <t>Yugo (yoke) estriado para cardán serie 330.</t>
+    <t>Horquilla del extremo del cardán que encaja en el eje estriado de la toma de fuerza o del implemento. Serie 330.</t>
   </si>
   <si>
     <t>CC56.jpeg</t>
@@ -183,7 +183,7 @@
     <t>Cruceta 30 x 106</t>
   </si>
   <si>
-    <t>Cruceta Aemco 30 x 106.</t>
+    <t>Pieza en cruz que articula las horquillas del cardán y le permite girar en ángulo sin perder fuerza. Medida 30 x 106, original Aemco.</t>
   </si>
   <si>
     <t>CC55.jpeg</t>
@@ -195,7 +195,7 @@
     <t>Tubo cuadrado para cardán, cruceta 27 x 1,20 m</t>
   </si>
   <si>
-    <t>Tubo cuadrado de 1,20 m para cardán con cruceta 27.</t>
+    <t>Tubo exterior del cardán: junto con la barra cuadrada deja que el cardán se alargue o se acorte al subir y bajar el implemento. 1,20 m, para cruceta 27.</t>
   </si>
   <si>
     <t>CC28J-1200.jpeg</t>
@@ -207,7 +207,7 @@
     <t>Barra cuadrada para cardán, cruceta 27 x 1,20 m</t>
   </si>
   <si>
-    <t>Barra cuadrada de 1,20 m para cardán con cruceta 27.</t>
+    <t>Barra interior que se desliza dentro del tubo cuadrado del cardán y transmite el giro. 1,20 m, para cruceta 27.</t>
   </si>
   <si>
     <t>CC29A-1200.jpeg</t>
@@ -228,7 +228,7 @@
     <t>Abonadoras Vicon</t>
   </si>
   <si>
-    <t>Trompo para abonadora Vicon.</t>
+    <t>Repuesto del mecanismo de distribución de la abonadora, que esparce el fertilizante sobre el terreno. Original Vicon.</t>
   </si>
   <si>
     <t>22300.jpeg</t>
@@ -240,7 +240,7 @@
     <t>Péndulo</t>
   </si>
   <si>
-    <t>Péndulo para abonadora Vicon.</t>
+    <t>Tubo que oscila de lado a lado en la abonadora y lanza el fertilizante o la semilla para repartirlo de forma pareja. Original Vicon.</t>
   </si>
   <si>
     <t>07665.png</t>
@@ -252,7 +252,7 @@
     <t>Escala</t>
   </si>
   <si>
-    <t>Escala para abonadora Vicon.</t>
+    <t>Regula la abertura de salida de la abonadora para fijar cuánto fertilizante se reparte. Original Vicon.</t>
   </si>
   <si>
     <t>52429.jpeg</t>
@@ -264,7 +264,7 @@
     <t>Campana</t>
   </si>
   <si>
-    <t>Campana para abonadora Vicon.</t>
+    <t>Pieza de la abonadora por donde el fertilizante baja de la tolva hacia el mecanismo de distribución. Original Vicon.</t>
   </si>
   <si>
     <t>70632.jpeg</t>
@@ -282,7 +282,7 @@
     <t>Lumagi</t>
   </si>
   <si>
-    <t>Engrasadora de 12 kg con bajante, original Lumagi.</t>
+    <t>Engrasadora de 12 kg con manguera bajante para engrasar crucetas, rodamientos y puntos de lubricación de tractores e implementos. Original Lumagi.</t>
   </si>
   <si>
     <t>LUB600.jpeg</t>

</xml_diff>